<commit_message>
Actualització minutes + PwP Enric
</commit_message>
<xml_diff>
--- a/others/BURNDOWN-CHART.xlsx
+++ b/others/BURNDOWN-CHART.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enric/Documents/UNI Informatica/3r - Q2/E.Software/Projecte/others/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2E53B8D-9246-844F-9385-87794C27646A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F73D10F9-0A49-4F47-BB8E-C24A81E8A1D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -85,7 +85,7 @@
     <t>QUEMENGES</t>
   </si>
   <si>
-    <t>3.0</t>
+    <t>4.0</t>
   </si>
 </sst>
 </file>
@@ -645,25 +645,25 @@
                   <c:v>17</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>17</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>17</c:v>
+                  <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>17</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>17</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>17</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>17</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>17</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -727,25 +727,25 @@
                   <c:v>18.5</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>18.5</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>18.5</c:v>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>18.5</c:v>
+                  <c:v>8.5</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>18.5</c:v>
+                  <c:v>6.5</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>18.5</c:v>
+                  <c:v>6.5</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>18.5</c:v>
+                  <c:v>6.5</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>18.5</c:v>
+                  <c:v>6.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1707,15 +1707,19 @@
       <c r="B15" s="15">
         <v>9</v>
       </c>
-      <c r="C15" s="16"/>
-      <c r="D15" s="17"/>
+      <c r="C15" s="16">
+        <v>3</v>
+      </c>
+      <c r="D15" s="17">
+        <v>3.5</v>
+      </c>
       <c r="E15" s="20">
         <f t="shared" ref="E15:F15" si="8">E14-C15</f>
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F15" s="21">
         <f t="shared" si="8"/>
-        <v>18.5</v>
+        <v>15</v>
       </c>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
@@ -1743,15 +1747,19 @@
       <c r="B16" s="15">
         <v>10</v>
       </c>
-      <c r="C16" s="16"/>
-      <c r="D16" s="17"/>
+      <c r="C16" s="16">
+        <v>3</v>
+      </c>
+      <c r="D16" s="17">
+        <v>3</v>
+      </c>
       <c r="E16" s="20">
         <f t="shared" ref="E16:F16" si="9">E15-C16</f>
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F16" s="21">
         <f t="shared" si="9"/>
-        <v>18.5</v>
+        <v>12</v>
       </c>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
@@ -1779,15 +1787,19 @@
       <c r="B17" s="15">
         <v>11</v>
       </c>
-      <c r="C17" s="16"/>
-      <c r="D17" s="17"/>
+      <c r="C17" s="16">
+        <v>4</v>
+      </c>
+      <c r="D17" s="17">
+        <v>3.5</v>
+      </c>
       <c r="E17" s="20">
         <f t="shared" ref="E17:F17" si="10">E16-C17</f>
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="F17" s="21">
         <f t="shared" si="10"/>
-        <v>18.5</v>
+        <v>8.5</v>
       </c>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
@@ -1815,15 +1827,19 @@
       <c r="B18" s="15">
         <v>12</v>
       </c>
-      <c r="C18" s="16"/>
-      <c r="D18" s="17"/>
+      <c r="C18" s="16">
+        <v>2</v>
+      </c>
+      <c r="D18" s="17">
+        <v>2</v>
+      </c>
       <c r="E18" s="20">
         <f t="shared" ref="E18:F18" si="11">E17-C18</f>
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="F18" s="21">
         <f t="shared" si="11"/>
-        <v>18.5</v>
+        <v>6.5</v>
       </c>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
@@ -1855,11 +1871,11 @@
       <c r="D19" s="17"/>
       <c r="E19" s="20">
         <f t="shared" ref="E19:F19" si="12">E18-C19</f>
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="F19" s="21">
         <f t="shared" si="12"/>
-        <v>18.5</v>
+        <v>6.5</v>
       </c>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
@@ -1891,11 +1907,11 @@
       <c r="D20" s="17"/>
       <c r="E20" s="20">
         <f t="shared" ref="E20:F20" si="13">E19-C20</f>
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="F20" s="21">
         <f t="shared" si="13"/>
-        <v>18.5</v>
+        <v>6.5</v>
       </c>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
@@ -1927,11 +1943,11 @@
       <c r="D21" s="17"/>
       <c r="E21" s="20">
         <f t="shared" ref="E21:F21" si="14">E20-C21</f>
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="F21" s="21">
         <f t="shared" si="14"/>
-        <v>18.5</v>
+        <v>6.5</v>
       </c>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>

</xml_diff>